<commit_message>
Feat : Filled to Location code
</commit_message>
<xml_diff>
--- a/Data.xlsx
+++ b/Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://deltao365-my.sharepoint.com/personal/thisuwan_deltaww_com/Documents/Attachments/FillForm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://deltao365-my.sharepoint.com/personal/thisuwan_deltaww_com/Documents/Code/AutoRepairForm/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{6CCFAEFD-D040-48F4-A9B0-2689C74F0348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CD996947-84BD-4980-A712-417D5D3F2C0A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{CD996947-84BD-4980-A712-417D5D3F2C0A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>